<commit_message>
fix: remove PAGE_SIZE - all rows in HTML; add Week 15 inventory+sales+AMS data
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week14.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week14.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\ams_weekly_data\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1731C976-1305-4B7B-BEED-452439283C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E612C6C1-2F9B-41D5-8EC9-0E534D64DB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C2EB3544-0B30-4B5A-9817-98DE85FBF6BC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{C2EB3544-0B30-4B5A-9817-98DE85FBF6BC}"/>
   </bookViews>
   <sheets>
     <sheet name="SP" sheetId="1" r:id="rId1"/>

</xml_diff>